<commit_message>
atv2 juiz online 70 bi parametros
</commit_message>
<xml_diff>
--- a/dataset_m2.xlsx
+++ b/dataset_m2.xlsx
@@ -431,6 +431,313 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Question 77.1 (MC-NJ) - Step 3
+A 34-year-old woman comes to the office because of a 3- to 4-week history
+of swelling of her legs and a 9-kg (20-lb) weight
+gain. Medical history is significant for sickle cell trait and mild anemia. She
+has been taking 800 mg of ibuprofen three times
+daily for Achilles tendinitis diagnosed 1 month ago. She has smoked five
+cigarettes daily for the past 15 years, and she drinks
+one to five beers on weekends. She experimented with cocaine briefly 16
+years ago, but she has never used intravenous
+drugs. She has been in a monogamous sexual relationship for the past 12
+years. Today, vital signs are temperature
+37.2°C (99.0°F), pulse 88/min, respirations 16/min, and blood pressure
+145/95 mm Hg. Physical examination discloses
+periorbital edema but no jugular venous distention. Lungs are clear to
+auscultation. Cardiac examination discloses an S1 and
+S2 without murmurs or gallops. Abdominal examination discloses bulging
+flanks and shifting dullness to percussion.
+Examination of the lower extremities shows pitting edema from the mid
+thigh to the ankles bilaterally. Results of which of
+the following studies are most likely to be abnormal in this patient?
+(A) Echocardiography
+(B) HIV antibody study
+(C) Serum B-type natriuretic peptide concentration
+(D) Toxicology screening of the urine
+(E) Urine protein concentration</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Question 78.1 (MC-NJ) - Step 3
+A 54-year-old woman comes to the office because she has had intermittent
+shooting pain over her right cheek and jaw during
+the past 3 weeks. Each episode of pain lasts for 1 second or less. The pain is
+often triggered by cold air, chewing, tactile
+stimulation, and brushing her teeth. She has had no trauma to the face or
+head. Medical history is remarkable for tension
+headaches, obesity, and gastric bypass surgery. She is 165 cm (5 ft 5 in) tall
+and weighs 62 kg (137 lb); BMI is 23 kg/m². Vital signs are normal. The
+patient cannot tolerate touch over the right side of the face. There is no
+facial weakness or loss of
+sensation. The remainder of the physical examination shows no
+abnormalities. CT scan of the head with and without contrast
+shows no abnormalities. Which of the following is the most appropriate
+pharmacotherapy at this time?
+(A) Carbamazepine
+(B) Lamotrigine
+(C) Levetiracetam
+(D) Topiramate
+(E) Zonisamide</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Question 79.1 (MC-NJ) - Step 3
+A 25-year-old man, who was admitted to the hospital 5 hours ago because
+of nausea, light-headedness, and muscle aches that
+began after he completed a marathon, now reports worsening pain in his
+right leg. On admission, the patient reported only
+mild muscle aching, but he now rates the pain in his right lower extremity
+as a 9 on a 10-point scale. Laboratory studies on
+admission were notable for a serum creatine kinase concentration of
+10,000 U/L and a serum creatinine concentration of 1.7
+mg/dL. Since admission the patient has received 5 L of 0.9% saline and his
+nausea and light-headedness have resolved. He is
+alert and fully oriented. Vital signs are temperature 36.9°C (98.5°F), pulse
+88/min, respirations 16/min, and blood pressure
+126/82 mmHg. Pulse oximetry on room air shows an oxygen saturation of
+97%. Cardiopulmonary and abdominal
+examinations disclose no abnormalities. Passive flexion of the toes elicits
+pain over the anterior portion of the right lower
+extremity below the knee. Distal pulses are present in the lower
+extremities bilaterally. The remainder of the physical
+examination discloses no abnormalities. Results of laboratory studies
+obtained 1 hour ago are shown:
+Serum:
+Urea nitrogen 12 mg/dL
+Creatinine 1.2 mg/dL
+Na+ 140 mEq/L
+K+ 4.0 mEq/L
+Cl− 100 mEq/L
+HCO3 −24 mEq/L
+Blood:
+Hemoglobin 14.0 g/dL
+WBC 14,000/mm3
+Neutrophils, segmented 60%
+Which of the following is the most appropriate next step in management?
+(A) Application of ice to the right lower extremity
+(B) Cyclobenzaprine therapy
+(C) Measurement of lower extremity compartment pressures
+(D) MRI of the right lower extremity
+(E) Nonsteroidal anti-inflammatory drug therapy</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Question 80.1 (MC-NJ) - Step 3
+A 9-year-old boy is brought to the office by his parents to establish care
+after recently moving to the area. The patient has not
+been evaluated by a physician in 4 years. He has been generally healthy.
+Medical history is significant for pneumonia at age
+3 years. He takes no medications. He is at the 25th percentile for height,
+weight, and BMI. Vital signs are temperature
+37.0°C (98.6°F), pulse 82/min, respirations 20/min, and blood pressure
+112/74 mm Hg. Cardiac examination discloses a
+grade 3/6 systolic murmur audible along the left sternal border at the third
+and fourth intercostal spaces. Femoral pulses are
+weak and brachial pulses are strong; there is a radiofemoral delay. Chest x-
+ray discloses mild cardiomegaly with left
+ventricular prominence. ECG shows left ventricular hypertrophy. This
+patient is at greatest risk for which of the following
+complications?
+(A) Atrial fibrillation
+(B) Cor pulmonale
+(C) Systemic hypertension
+(D) Tricuspid valve regurgitation</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Question 81.1 (MC-NJ) - Step 3
+A 25-year-old woman comes to the office because of a 2-day history of
+right lower quadrant abdominal pain and vaginal
+spotting. She describes the abdominal pain as cramping and rates it as a 4
+on a 10-point scale. Medical history is
+unremarkable and the patient takes no medications. Menses are typically
+irregular but she thinks her last menstrual period
+was approximately 5 weeks ago. She is sexually active with one male
+partner and they use condoms occasionally. Vital signs
+are temperature 37.2°C (99.0°F), pulse 90/min, respirations 16/min, and
+blood pressure 110/65 mm Hg. Abdominal
+examination discloses tenderness to palpation of the right lower quadrant.
+Pelvic examination discloses dark blood in the
+vaginal vault. Hematocrit is 36%. Urine pregnancy test is positive. Pelvic
+ultrasonography shows a thickened endometrial
+lining and no adnexal masses. Which of the following is the most
+appropriate next step in management?
+(A) Admission to the hospital for observation
+(B) Diagnostic laparoscopy
+(C) Dilatation and curettage
+(D) Follow-up pelvic ultrasonography in 1 week
+(E) Serial serum β-hCG concentrations</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Question 82.1 (MC-NJ) - Step 3
+A 32-year-old woman, gravida 4, para 4, comes to the office 1 week after an
+uncomplicated vaginal delivery of a 3020-g (6-lb
+11-oz) term female newborn. She has been breast-feeding her daughter
+since birth. The patient says that she cries frequently
+for no reason, is irritable, and is worried about her infant's long-term
+health. The patient reports having no appetite. She says
+that her husband and mother say that she is depressed and think she is
+anorexic. She has not had auditory hallucinations,
+confusion, or disorientation. She denies suicidal or homicidal ideation. She
+has a history of postpartum psychosis following
+the birth of her first child; she had no similar symptoms after the births of
+her second and third children. Which of the
+following factors in this patient's history most strongly indicates a poor
+prognosis?
+(A) Anorexia
+(B) Depressed mood
+(C) History of psychosis
+(D) Multiparity</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Question 83.1 (MC-NJ) - Step 3
+A 47-year-old man comes to the office to establish care. He recently moved
+to the area and has not been evaluated by a
+physician for more than 3 years. He reports a 1-year history of bilateral
+knee pain that worsens after prolonged standing, but
+he otherwise has felt well. Medical history is unremarkable and his only
+medication is acetaminophen as needed for his knee
+pain. Family history is significant for hypothyroidism in his mother and
+myocardial infarction in a paternal uncle at age
+55 years. The patient drinks five to six beers weekly and does not smoke
+cigarettes. BMI is 32 kg/m² . Vital signs are
+temperature 36.1°C (97.0°F), pulse 78/min, respirations 12/min, and blood
+pressure 138/89 mm Hg. The patient is not in
+distress. Physical examination discloses no abnormalities. Results of fasting
+serum lipid studies obtained in preparation for
+today's visit are shown:
+Cholesterol
+Total 264 mg/dL
+HDL 54 mg/dL
+LDL 170 mg/dL
+Triglycerides 200 mg/dL
+Which of the following is the most appropriate next step in management
+regarding the patient's laboratory study results?
+(A) Prescribe atorvastatin
+(B) Prescribe cholestyramine
+(C) Recommend diet and low-impact exercise
+(D) Refer the patient to a cardiologist
+(E) Repeat fasting laboratory studies in 1 month</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Question 84.1 (MC-NJ) - Step 3
+A 37-year-old man comes to the emergency department because he has
+felt nauseated and light-headed for the past hour.
+Medical history is significant for esophageal varices secondary to alcohol-
+related cirrhosis and ascites treated with
+spironolactone. He drinks eight to ten alcoholic beverages daily. While you
+are obtaining additional history, the patient
+vomits a large volume of bright red blood and becomes difficult to arouse.
+Vital signs are temperature 36.0°C (96.8°F), pulse
+110/min, respirations 12/min, and blood pressure 90/50 mm Hg. Following
+initiation of intravenous fluids, which of the
+following is the most appropriate immediate management?
+(A) Arrange for transjugular intrahepatic portal vein shunting
+(B) Begin intravenous vasopressin therapy
+(C) Do endotracheal intubation
+(D) Do upper endoscopy
+(E) Insert an esophageal tube for balloon tamponade</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Question 85.1 (MC-NJ) - Step 3
+A 25-year-old man was admitted to the hospital yesterday with a massive
+hemothorax sustained as a result of a stab wound. Left lateral thoracotomy
+was done because more than 2 L of blood returned following chest tube
+placement. The thoracotomy disclosed a bleeding intercostal vessel that
+was repaired by suture ligation. Vital signs now are temperature 36.0°C
+(96.8°F), pulse 100/min, respirations 18/min, and blood pressure 120/78
+mm Hg. Pulse oximetry on 5 L/min of oxygen via nasal cannula shows an
+oxygen saturation of 95%. Physical examination discloses a well-
+approximated staple line at the incision site and mild erythema. Decreased
+respiratory excursion is noted on the left side. The chest tube is draining a
+small amount of serosanguineous fluid; no air leak is noted. Which of the
+following is the most appropriate next step in management? Why not the
+other choices?
+(A) Administration of broad-spectrum antibiotics
+(B) Initiation of tube feedings
+(C) Pain reduction
+(D) Physical therapy
+(E) Psychological evaluation for post-traumatic stress disorder</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Question 86.1 (MC-NJ) - Step 3
 A 45-year-old man returns to the office for ongoing treatment of
 tuberculous pericarditis. Pericardiocentesis 9 weeks ago
@@ -459,14 +766,14 @@
 (E) Order echocardiography</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Question 87.1 (MC-NJ) - Step 3
 A 40-year-old woman, gravida 2 para 2, comes to the office because of
@@ -487,14 +794,14 @@
 (E) Warfarin therapy</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Question 89.1 (MC-NJ) - Step 3
 A 39-year-old woman, gravida 2, para 2, comes to the community-based
@@ -519,14 +826,14 @@
 (E) Stage of disease</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>Question 90.1 (MC-NJ) - Step 3
 A 28-year-old man comes to the office for an annual health maintenance
@@ -560,14 +867,14 @@
 (E) Suppressing appetite</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Question 91.1 (MC-NJ) - Step 3
 A 22-year-old man comes to the office for evaluation 3 days after his
@@ -589,14 +896,14 @@
 (E) Reassure the patient that no treatment is necessary</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Question 92.1 (MC-NJ) - Step 3
 A 25-year-old man comes to the office because he has had a "coating" on
@@ -633,14 +940,14 @@
 (E) Systemic chemotherapy with liposomal doxorubicin</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Question 93.1 (MC-NJ) - Step 3
 A 24-year-old recent college graduate comes to the office because of a 3-
@@ -661,14 +968,14 @@
 (E) Reassure the patient that her symptoms will resolve in time</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Question 94.1 (MC-NJ) - Step 3
 A 22-year-old woman comes to the emergency department because of a 5-
@@ -691,14 +998,14 @@
 (E) Tonsillectomy</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Question 95.1 (MC-NJ) - Step 3
 A 26-year-old man, who is admitted to the hospital to undergo
@@ -720,14 +1027,14 @@
 disorder</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Question 97.1 (MC-NJ) - Step 3
 A 29-year-old woman, gravida 3, para 3, comes to the office because of a 1-
@@ -747,14 +1054,14 @@
 (E) Recommend decreasing physical activity</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>Question 98.1 (MC-NJ) - Step 3
 A 46-year-old woman comes to the office because of a 4-month history of
@@ -777,14 +1084,14 @@
 (E) Trial of hormone replacement therapy</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>Question 99.1 (MC-NJ) - Step 3
 A 36-year-old woman is referred to the office for evaluation of a fasting
@@ -809,14 +1116,14 @@
 (E) Strict low-fat diet</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>Question 100.1 (MC-NJ) - Step 3
 A 57-year-old man was admitted to the intensive care unit from the
@@ -847,14 +1154,14 @@
 (F) Needle decompression</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>Question 101.1 (MC-NJ) - Step 3
 A 32-year-old woman comes to the office because of a 2-week history of
@@ -876,14 +1183,14 @@
 (E) Sclerotherapy</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Question 103.1 (MC-NJ) - Step 3
 A 16-year-old girl is brought to the office by her mother because she is
@@ -905,14 +1212,14 @@
 (E) Assure the patient that no anti-infective prophylaxis is necessary</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>Question 104.1 (MC-NJ) - Step 3
 A 27-year-old nulligravid woman comes to the office because of a 1-month
@@ -945,14 +1252,14 @@
 (E) Transfusion of packed red blood cells</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t>Question 105.1 (MC-NJ) - Step 3
 A 67-year-old man with Parkinson disease is admitted to the hospital for
@@ -981,14 +1288,14 @@
 (E) Prescribe prophylactic levofloxacin</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>Question 106.1 (MC-NJ) - Step 3
 A 47-year-old man is admitted to the hospital through the emergency
@@ -1011,343 +1318,6 @@
 (E) Metoprolol</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Question 107.1 (MC-NJ) - Step 3
-A 23-year-old man comes to the clinic to establish care after moving to the
-area for his first job since graduating from college. He has felt well. Medical
-history is remarkable for Hodgkin lymphoma diagnosed 10 years ago, which
-was treated with radiation therapy and a chemotherapy regimen of
-vinblastine, doxorubicin, methotrexate, and prednisone. BMI is 20 kg/m².
-Vital signs are within normal limits. The patient appears well. Physical
-examination discloses no abnormalities. Which of the following screening
-studies is most appropriate to include in this patient's annual
-examinations?
-(A) Bone marrow aspiration and complete blood count
-(B) CT scan of the chest, abdomen, and pelvis
-(C) Echocardiography
-(D) Fine-needle aspiration biopsy of the thyroid gland
-(E) Nerve conduction studies</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Question 108.1 (MC-NJ) - Step 3
-A 5-year-old boy returns to the office with his mother to discuss results of
-studies done to evaluate his behavior of eating dirt. The patient sits quietly
-while his mother answers questions about his health. She says her son
-seems healthy, although he does not seem to be as active as other children
-his age. He has said his head hurts three or four times during the past 2
-weeks. He has not had fever, sweats, or chills. She says he has a good
-appetite but has had a habit of eating sand and dirt since age 3 years. She
-says, "I don't know where he gets that habit. I used to eat dirt, but I stopped
-years ago. I try to stop him from eating dirt, but I'm not around much since
-I work two jobs." The patient takes no medications. Vaccinations are up-to-
-date. Height, weight, and BMI are at the 50th percentile. Vital signs are
-normal. Physical examination discloses no abnormalities except for
-symmetrical nontender cervical adenopathy. Results of laboratory studies,
-including serum zinc, lead, and iron concentrations, are within the
-reference ranges. Serologic testing confirms toxoplasmosis. In addition to
-prescribing pyrimethamine and sulfadiazine therapy, which of the following
-is the most appropriate next step in management?
-(A) Prescribe fluoxetine
-(B) Prescribe methylphenidate
-(C) Prescribe risperidone
-(D) Refer the patient to a child psychiatrist
-(E) Refer the patient to a dietician</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Question 109.1 (MC-NJ) - Step 3
-A 55-year-old woman is brought to the office by her husband because of
-increasingly severe pain in her mid back for the past week. She says the
-pain is especially severe with walking. Her husband says she has been
-favoring her right leg for the past 3 days. Ibuprofen no longer controls the
-pain. She enjoys gardening but had to discontinue it 1 week ago because of
-the pain. She has not had bowel or bladder dysfunction. She underwent a
-right mastectomy 3 years ago for carcinoma and has been taking tamoxifen
-since that time. She is 173 cm (5 ft 8 in) tall and weighs 66 kg (145 lb); BMI is
-22 kg/m². Vital signs are temperature 38.0°C (100.4°F), pulse 90/min,
-respirations 15/min, and blood pressure 118/72 mm Hg. Strength is 3/5 in
-all muscle groups of the right lower extremity and 5/5 in the left lower
-extremity. Achilles and patellar reflexes are hyperactive on the right and
-normal on the left. Sensation to pinprick and temperature is decreased in
-the left lower extremity to the level of the inguinal ligament. Sensation to
-vibration is decreased in the right lower extremity. Reflexes and sensation
-are otherwise intact. Rectal sphincter tone is normal. Which of the
-following is the most appropriate next step?
-(A) Acetaminophen-oxycodone therapy and referral for physical therapy
-(B) Admission to the hospital for pain control
-(C) Electromyography and nerve conduction studies
-(D) MRI of the thoracic spine
-(E) Technetium 99m scan</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Question 110.1 (MC-NJ) - Step 3
-A 7-year-old boy with sickle cell disease is brought to the office by his
-father because of fever and bone pain. The father says that his son was
-discharged 5 days ago after a 3-day hospitalization for the same symptoms.
-The patient had been admitted with a diagnosis of vaso-occlusive crisis
-with bone infarct, with resolution of symptoms after treatment with
-intravenous fluids, narcotics, and antibiotic therapy for 3 days. Blood
-cultures were negative. The patient's back pain and fever recurred 2 days
-ago and seem more severe than prior to the hospitalization. His medical
-chart shows that he had one other uncomplicated hospital admission at
-age 4 years for a vaso-occlusive crisis with lower extremity bone pain. Vital
-signs today are temperature 39.2°C (102.5°F), pulse 110/min, respirations
-24/min, and blood pressure 115/60 mm Hg. The patient is uncomfortable
-but does not appear toxic. Cardiac examination discloses a grade 2/6
-systolic ejection murmur at the left lower sternal border. Spleen is not
-palpated. There is considerable tenderness over the L1–L3 region of the
-back without fluctuation. There is diffuse pain in both thighs without
-localization, but range of motion is normal. Which of the following studies
-is most likely to establish the diagnosis at this time?
-(A) Blood culture
-(B) CT scan of the spine
-(C) MRI of the lumbar spine
-(D) Ultrasonography of the spine
-(E) X-ray of the spine</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Question 111.1 (MC-NJ) - Step 3
-A 7-year-old boy with sickle cell disease is brought to the office by his
-father because of fever and bone pain. The father says that his son was
-discharged 5 days ago after a 3-day hospitalization for the same symptoms.
-The patient had been admitted with a diagnosis of vaso-occlusive crisis
-with bone infarct, with resolution of symptoms after treatment with
-intravenous fluids, narcotics, and antibiotic therapy for 3 days. Blood
-cultures were negative. The patient's back pain and fever recurred 2 days
-ago and seem more severe than prior to the hospitalization. His medical
-chart shows that he had one other uncomplicated hospital admission at
-age 4 years for a vaso-occlusive crisis with lower extremity bone pain. Vital
-signs today are temperature 39.2°C (102.5°F), pulse 110/min, respirations
-24/min, and blood pressure 115/60 mm Hg. The patient is uncomfortable
-but does not appear toxic. Cardiac examination discloses a grade 2/6
-systolic ejection murmur at the left lower sternal border. Spleen is not
-palpated. There is considerable tenderness over the L1–L3 region of the
-back without fluctuation. There is diffuse pain in both thighs without
-localization, but range of motion is normal.
-MRI of the spine confirms the diagnosis. Which of the following is the most
-appropriate initial intravenous pharmacotherapy?
-(A) Ceftriaxone
-(B) Cephalothin and clarithromycin
-(C) Clindamycin and gentamicin
-(D) Nafcillin
-(E) Vancomycin and cefotaxime</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Question 112.1 (MC-NJ) - Step 3
-A 24-year-old man comes to the emergency department because of right
-lower quadrant abdominal pain and nausea that began suddenly 6 hours
-ago. He rates the pain as a 6 on a 10-point scale and asks for pain
-medication. Medical history is unremarkable. He takes only a multivitamin.
-Vital signs on arrival are temperature 38.7°C (101.6°F), pulse 105/min,
-respirations 16/min, and blood pressure 110/85 mm Hg. Physical
-examination discloses exquisite tenderness in the right lower quadrant of
-the abdomen. The remainder of the examination discloses no
-abnormalities. The surgical consultant cannot evaluate the patient for 2
-hours. Which of the following is the most appropriate next step?
-(A) Administer acetaminophen
-(B) Administer gabapentin
-(C) Administer lorazepam
-(D) Administer morphine
-(E) Explain to the patient that analgesics would interfere with the surgical
-examination</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Question 114.1 (MC-NJ) - Step 3
-A 74-year-old man who had a stroke 2 years ago is admitted to the hospital
-from the nursing care facility because of a 4-day history of reduced urinary
-output, and worsening abdominal pain, nausea, and lethargy. The stroke
-had resulted in right-sided hemiparesis and difficulties with speech and
-swallowing. Medical history is also significant for hypertension. The patient
-has been hospitalized twice during the past 3 months for pneumonias that
-did not respond to oral antibiotic therapy in the nursing facility. He
-underwent bladder catheterization during each of the recent
-hospitalizations for a total of 6 days to monitor urine output. The catheter
-was removed prior to each discharge. Bladder catheterization attempts
-during the past several days in response to his current symptoms have
-been unsuccessful. Now on admission, the patient appears agitated and
-confused. Vital signs are temperature 36.9°C (98.4°F), pulse 110/min,
-respirations 24/min, and blood pressure 160/100 mm Hg. Physical
-examination discloses jugular venous distention, 8 cm at 45 degrees. Lungs
-are clear to auscultation. Auscultation of the heart discloses regular
-tachycardia with no gallops. There is fullness and tenderness to palpation
-of the low central abdomen but no rebound or guarding. Examination of
-the extremities shows 1+ pedal edema bilaterally. The prostate is normal in
-size and has no palpable nodules or tenderness. Results of laboratory
-studies are shown:
-Serum
-Urea nitrogen - 73 mg/dL
-Creatinine - 4.2 mg/dL
-Calcium - 8.6 mg/dL
-Na⁺ - 134 mEq/L
-K⁺ - 5.6 mEq/L
-Cl⁻ - 100 mEq/L
-HCO3⁻ - 20 mEq/L
-Mg2⁺ - 2.0 mEq/L
-Glucose - 126 mg/dL
-Phosphorus - 4.8 mEq/L
-Blood
-Hematocrit - 32%
-Hemoglobin - 10.6 g/dL
-WBC - 8200/mm³
-Platelet count - 359,000/mm³
-Ultrasonography shows distention of the bladder and bilateral
-hydronephrosis. ECG shows sinus tachycardia. Which of the following is
-the most appropriate next step?
-(A) Administration of bethanechol
-(B) Administration of prazosin
-(C) Hemodialysis
-(D) Placement of a suprapubic catheter
-(E) Ultrafiltration</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Question 115.1 (MC-NJ) - Step 3
-A 47-year-old man comes to the emergency department because of a 3-day
-history of increasing pain, tenderness, and swelling near the fingernail of
-his right index finger. He rates the pain as an 8 on a 10-point scale. He has
-not had fever or chills, and he has not sustained any trauma to the finger.
-Medical history is unremarkable and the patient takes no medications. He
-appears generally well and is not in distress. Vital signs are temperature
-37.1°C (98.8°F), pulse 72/min, respirations 14/min, and blood pressure
-120/80 mm Hg. Physical examination of the right hand discloses swelling,
-erythema, warmth, and tenderness of the periungual region of the right
-index finger. There is a mildly fluctuant area near the nail edge. The
-remainder of the physical examination discloses no abnormalities. Which
-of the following is the most appropriate next step in management?
-(A) Incision and drainage
-(B) Oral cefazolin therapy
-(C) Topical neomycin therapy
-(D) Warm-water soaks</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Question 116.1 (MC-NJ) - Step 3
-A 12-year-old girl with type 1 diabetes mellitus is brought to the emergency
-department by her parents because of a 2-day history of nausea, vomiting,
-and decreased oral intake. Medications are insulin glargine and insulin
-aspart. She decreased her insulin dose at the onset of symptoms but her
-condition has since worsened and she now is unable to consume solids or
-liquids without subsequent vomiting. She reports feeling dizzy on standing.
-Medical history is otherwise unremarkable. She is at the 50th percentile for
-height, weight, and BMI. Vital signs are temperature 37.8°C (100.1°F), pulse
-118/min, respirations 27/min, and blood pressure 85/47 mm Hg. Pulse
-oximetry on room air shows an oxygen saturation of 99%. Physical
-examination discloses dry mucous membranes, delayed capillary refill time,
-and poor skin turgor. Palpation of the abdomen discloses diffuse
-tenderness with no rebound or guarding. The remainder of the physical
-examination discloses no abnormalities. Results of laboratory studies
-obtained on arrival are shown:
-Serum
-Urea nitrogen - 28 mg/dL
-Creatinine - 1.2 mg/dL
-Na⁺ - 126 mEq/L
-K⁺ - 4.3 mEq/L
-Cl⁻ - 95 mEq/L
-HCO3⁻ - 9 mEq/L
-Glucose - 563 mg/dL
-Arterial blood gas values on room air
-HCO3⁻ 10 mEq/L
-Partial Pressure of Oxygen - 98 mm Hg
-Partial Pressure of Carbon Dioxide - 22 mm Hg
-pH - 7.20
-Boluses of intravenous 0.9% saline are administered and an infusion of
-insulin is initiated. Three hours later the patient becomes somnolent and
-develops a headache. She has had one episode of emesis and one episode
-of incontinence. Her urine output has been 30 mL/h. Results of follow-up
-serum laboratory studies are shown:
-Urea nitrogen - 24 mg/dL
-Creatinine - 1.1 mg/dL
-Na⁺ - 127 mEq/L
-K⁺ - 3.7 mEq/L
-Cl⁻ - 98 mEq/L
-HCO3⁻ - 11 mEq/L
-Glucose - 287 mg/dL
-Which of the following is the most appropriate intravenous
-pharmacotherapy?
-(A) Bicarbonate
-(B) Dexamethasone
-(C) 50% Dextrose
-(D) Furosemide
-(E) Mannitol</t>
-        </is>
-      </c>
       <c r="B28" t="inlineStr">
         <is>
           <t>E</t>

</xml_diff>